<commit_message>
relatorio excel dias 09 e 10 de maio
</commit_message>
<xml_diff>
--- a/saida_skus/SKU_BRINQ-001-BINGO-48-CARTELAS.xlsx
+++ b/saida_skus/SKU_BRINQ-001-BINGO-48-CARTELAS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analise" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,11 +33,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00008000"/>
+      <color rgb="00D93025"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00D93025"/>
+      <color rgb="00008000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O77"/>
+  <dimension ref="A1:O83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -559,12 +559,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -589,33 +589,33 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>R$ 79,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>▲ 26,3%</t>
+          <t>▼ 34,5%</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>8,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L2" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>0,9%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -632,12 +632,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -662,33 +662,33 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>R$ 711,00</t>
+          <t>R$ 40,00</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>▲ 19,9%</t>
+          <t>▼ 49,4%</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>149</v>
+        <v>125</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>▼ 22,8%</t>
+          <t>▲ 290,6%</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>12,1%</t>
+          <t>0,8%</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>8,1%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -705,12 +705,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -735,33 +735,33 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>R$ 79,00</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>▼ 13,6%</t>
+          <t>▲ 38,1%</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>10,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -778,12 +778,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -808,33 +808,33 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>R$ 593,00</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>▲ 25,1%</t>
+          <t>R$ 79,00</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>▲ 97,5%</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>193</v>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>▲ 17,7%</t>
+        <v>32</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>▲ 966,7%</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>7,8%</t>
+          <t>6,3%</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>5,7%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -851,12 +851,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -881,33 +881,33 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>R$ 79,00</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 40,00</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>▼ 49,4%</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>21</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>▼ 12,5%</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>9,1%</t>
+          <t>4,8%</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -924,12 +924,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -954,33 +954,33 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>R$ 474,00</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>▼ 29,5%</t>
+          <t>R$ 40,00</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>▼ 94,4%</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>164</v>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>▼ 10,9%</t>
+        <v>3</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>▼ 98,0%</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>7,3%</t>
+          <t>33,3%</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -997,12 +997,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1032,20 +1032,20 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>▼ 26,7%</t>
+          <t>▲ 26,3%</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>9,1%</t>
+          <t>8,3%</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,9%</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1100,33 +1100,33 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>R$ 672,00</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>▲ 40,6%</t>
+          <t>R$ 711,00</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>▲ 19,9%</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>184</v>
+        <v>149</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>▲ 2,8%</t>
+          <t>▼ 22,8%</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>9,2%</t>
+          <t>12,1%</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>8,6%</t>
+          <t>8,1%</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1143,12 +1143,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1173,33 +1173,33 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 79,00</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>▲ 57,9%</t>
+          <t>▼ 13,6%</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>10,5%</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,8%</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1216,12 +1216,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1246,33 +1246,33 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>R$ 478,00</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>▲ 112,4%</t>
+          <t>R$ 593,00</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>▲ 25,1%</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>179</v>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>▲ 51,7%</t>
+        <v>193</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>▲ 17,7%</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>6,1%</t>
+          <t>7,8%</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>5,8%</t>
+          <t>5,7%</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1319,16 +1319,16 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+          <t>R$ 79,00</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>10,5%</t>
+          <t>9,1%</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>1,5%</t>
+          <t>0,8%</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1362,12 +1362,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1392,33 +1392,33 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>R$ 225,00</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>▼ 16,4%</t>
+          <t>R$ 474,00</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>▼ 29,5%</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>118</v>
+        <v>164</v>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>▲ 28,3%</t>
+          <t>▼ 10,9%</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>4,2%</t>
+          <t>7,3%</t>
         </is>
       </c>
       <c r="L13" s="2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>3,7%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1435,12 +1435,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1465,33 +1465,33 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+          <t>R$ 79,00</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>▼ 24,0%</t>
+        <v>22</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>▼ 26,7%</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>5,3%</t>
+          <t>9,1%</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1508,12 +1508,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1538,33 +1538,33 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>R$ 269,00</t>
+          <t>R$ 672,00</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>▼ 25,1%</t>
+          <t>▲ 40,6%</t>
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>▲ 10,8%</t>
+        <v>184</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>▲ 2,8%</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>5,4%</t>
+          <t>9,2%</t>
         </is>
       </c>
       <c r="L15" s="2" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>4,2%</t>
+          <t>8,6%</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1581,12 +1581,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1611,33 +1611,33 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>R$ 135,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>▲ 200,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>▲ 56,2%</t>
+        <v>30</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>▲ 57,9%</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>12,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L16" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>1,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1654,12 +1654,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1684,33 +1684,33 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>R$ 359,00</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>▲ 298,9%</t>
+          <t>R$ 478,00</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>▲ 112,4%</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>83</v>
+        <v>179</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>▼ 2,4%</t>
+          <t>▲ 51,7%</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>9,6%</t>
+          <t>6,1%</t>
         </is>
       </c>
       <c r="L17" s="2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>4,5%</t>
+          <t>5,8%</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1727,12 +1727,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1757,33 +1757,33 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
+          <t>R$ 90,00</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>▲ 23,1%</t>
-        </is>
-      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>6,3%</t>
+          <t>10,5%</t>
         </is>
       </c>
       <c r="L18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>1,5%</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1800,12 +1800,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1830,33 +1830,33 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>▼ 71,3%</t>
+          <t>R$ 225,00</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>▼ 16,4%</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>118</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>▲ 28,3%</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>2,4%</t>
+          <t>4,2%</t>
         </is>
       </c>
       <c r="L19" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>1,5%</t>
+          <t>3,7%</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -1873,12 +1873,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1906,22 +1906,22 @@
           <t>R$ 45,00</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>▼ 7,1%</t>
+        <v>19</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>▼ 24,0%</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>5,3%</t>
         </is>
       </c>
       <c r="L20" s="2" t="n">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,7%</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -1946,12 +1946,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1976,33 +1976,33 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>R$ 314,00</t>
+          <t>R$ 269,00</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>▲ 16,7%</t>
+          <t>▼ 25,1%</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>▲ 2,4%</t>
+        <v>92</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>▲ 10,8%</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>8,2%</t>
+          <t>5,4%</t>
         </is>
       </c>
       <c r="L21" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>4,2%</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2049,33 +2049,33 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
+          <t>R$ 135,00</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▲ 200,0%</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>▲ 16,7%</t>
+        <v>25</v>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>▲ 56,2%</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>7,1%</t>
+          <t>12,0%</t>
         </is>
       </c>
       <c r="L22" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>0,6%</t>
+          <t>1,7%</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -2092,12 +2092,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2122,33 +2122,33 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>R$ 269,00</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>▲ 19,6%</t>
+          <t>R$ 359,00</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>▲ 298,9%</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
         <v>83</v>
       </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>▼ 23,1%</t>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>▼ 2,4%</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>7,2%</t>
+          <t>9,6%</t>
         </is>
       </c>
       <c r="L23" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>3,7%</t>
+          <t>4,5%</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -2165,12 +2165,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2195,33 +2195,33 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
+          <t>R$ 45,00</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>▼ 25,0%</t>
+          <t>▲ 23,1%</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>16,7%</t>
+          <t>6,3%</t>
         </is>
       </c>
       <c r="L24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>1,3%</t>
+          <t>0,7%</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -2238,12 +2238,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2268,33 +2268,33 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>R$ 225,00</t>
+          <t>R$ 90,00</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>▲ 150,0%</t>
+          <t>▼ 71,3%</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>108</v>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>▲ 58,8%</t>
+        <v>85</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>2,4%</t>
         </is>
       </c>
       <c r="L25" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>1,5%</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -2311,12 +2311,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2341,33 +2341,33 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>▼ 5,9%</t>
+        <v>13</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>▼ 7,1%</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>7,7%</t>
         </is>
       </c>
       <c r="L26" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -2384,12 +2384,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2414,33 +2414,33 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 314,00</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>▲ 16,7%</t>
         </is>
       </c>
       <c r="I27" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>▲ 240,0%</t>
+        <v>85</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>▲ 2,4%</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>2,9%</t>
+          <t>8,2%</t>
         </is>
       </c>
       <c r="L27" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>1,5%</t>
+          <t>3,3%</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -2457,12 +2457,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2490,22 +2490,22 @@
           <t>R$ 45,00</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>▲ 21,4%</t>
+        <v>14</v>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>▲ 16,7%</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>5,9%</t>
+          <t>7,1%</t>
         </is>
       </c>
       <c r="L28" s="2" t="n">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
@@ -2530,12 +2530,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2560,33 +2560,33 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
+          <t>R$ 269,00</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>▼ 44,8%</t>
+          <t>▲ 19,6%</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>▼ 77,8%</t>
+        <v>83</v>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>▼ 23,1%</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>10,0%</t>
+          <t>7,2%</t>
         </is>
       </c>
       <c r="L29" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>0,9%</t>
+          <t>3,7%</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -2603,12 +2603,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2633,33 +2633,33 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>▼ 46,4%</t>
+          <t>R$ 90,00</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>▲ 16,7%</t>
+          <t>▼ 25,0%</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>7,1%</t>
+          <t>16,7%</t>
         </is>
       </c>
       <c r="L30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>1,3%</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
@@ -2676,12 +2676,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2706,33 +2706,33 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>R$ 163,00</t>
+          <t>R$ 225,00</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>▼ 65,5%</t>
+          <t>▲ 150,0%</t>
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>▼ 18,9%</t>
+          <t>▲ 58,8%</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>4,4%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="L31" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>2,5%</t>
+          <t>3,3%</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -2749,12 +2749,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2779,33 +2779,33 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>R$ 84,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>▲ 115,4%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>▲ 33,3%</t>
+          <t>▼ 5,9%</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>16,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L32" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>1,2%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -2822,12 +2822,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2852,33 +2852,33 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>R$ 473,00</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>▲ 140,1%</t>
+          <t>R$ 90,00</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>111</v>
+        <v>68</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>▼ 13,3%</t>
+          <t>▲ 240,0%</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>10,8%</t>
+          <t>2,9%</t>
         </is>
       </c>
       <c r="L33" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>6,8%</t>
+          <t>1,5%</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
@@ -2895,12 +2895,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2925,25 +2925,25 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>R$ 39,00</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>▼ 66,9%</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▲ 21,4%</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>11,1%</t>
+          <t>5,9%</t>
         </is>
       </c>
       <c r="L34" s="2" t="n">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>0,6%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -2968,12 +2968,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2998,33 +2998,33 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>R$ 197,00</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>▼ 58,4%</t>
+          <t>R$ 90,00</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>▼ 44,8%</t>
         </is>
       </c>
       <c r="I35" s="2" t="n">
-        <v>128</v>
+        <v>20</v>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>▲ 15,3%</t>
+          <t>▼ 77,8%</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>3,9%</t>
+          <t>10,0%</t>
         </is>
       </c>
       <c r="L35" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>2,8%</t>
+          <t>0,9%</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -3041,12 +3041,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3071,33 +3071,33 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>R$ 118,00</t>
+          <t>R$ 45,00</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>▲ 162,2%</t>
+          <t>▼ 46,4%</t>
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>14</v>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>▲ 16,7%</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>16,7%</t>
+          <t>7,1%</t>
         </is>
       </c>
       <c r="L36" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>1,5%</t>
+          <t>0,7%</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
@@ -3114,12 +3114,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3144,33 +3144,33 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>R$ 473,00</t>
+          <t>R$ 163,00</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>▲ 71,4%</t>
+          <t>▼ 65,5%</t>
         </is>
       </c>
       <c r="I37" s="2" t="n">
-        <v>111</v>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>90</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>▼ 18,9%</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>10,8%</t>
+          <t>4,4%</t>
         </is>
       </c>
       <c r="L37" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>5,9%</t>
+          <t>2,5%</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -3187,12 +3187,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3217,33 +3217,33 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 84,00</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>▲ 115,4%</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>12</v>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>▲ 33,3%</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>16,7%</t>
         </is>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>0,6%</t>
+          <t>1,2%</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -3260,12 +3260,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3290,33 +3290,33 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>R$ 276,00</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>▲ 249,4%</t>
+          <t>R$ 473,00</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>▲ 140,1%</t>
         </is>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>111</v>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>▼ 13,3%</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>10,8%</t>
         </is>
       </c>
       <c r="L39" s="2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>3,5%</t>
+          <t>6,8%</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3333,12 +3333,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3363,25 +3363,25 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+          <t>R$ 39,00</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,9%</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>9</v>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>11,1%</t>
         </is>
       </c>
       <c r="L40" s="2" t="n">
@@ -3406,12 +3406,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3436,33 +3436,33 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>R$ 79,00</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 197,00</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>▼ 58,4%</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>128</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>▲ 15,3%</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>4,0%</t>
+          <t>3,9%</t>
         </is>
       </c>
       <c r="L41" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>2,8%</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -3479,12 +3479,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3509,25 +3509,25 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>R$ 135,00</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
+          <t>R$ 118,00</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>▲ 162,2%</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I42" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>▼ 27,3%</t>
-        </is>
-      </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>18,8%</t>
+          <t>16,7%</t>
         </is>
       </c>
       <c r="L42" s="2" t="n">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>2,1%</t>
+          <t>1,5%</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3552,12 +3552,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3582,33 +3582,33 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>R$ 79,00</t>
+          <t>R$ 473,00</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>▼ 36,3%</t>
+          <t>▲ 71,4%</t>
         </is>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>111</v>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>10,8%</t>
         </is>
       </c>
       <c r="L43" s="2" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>1,2%</t>
+          <t>5,9%</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -3625,12 +3625,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3655,20 +3655,20 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3677,11 +3677,11 @@
         </is>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -3698,12 +3698,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3728,33 +3728,33 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>R$ 124,00</t>
+          <t>R$ 276,00</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>▼ 44,9%</t>
+          <t>▲ 249,4%</t>
         </is>
       </c>
       <c r="I45" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>▼ 29,1%</t>
+        <v>0</v>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>4,9%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L45" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>1,3%</t>
+          <t>3,5%</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -3771,12 +3771,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3804,22 +3804,22 @@
           <t>R$ 45,00</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>▼ 15,4%</t>
+        <v>0</v>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>9,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L46" s="2" t="n">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -3844,12 +3844,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3874,33 +3874,33 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>R$ 225,00</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>▼ 16,4%</t>
+          <t>R$ 79,00</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I47" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t>▲ 1,2%</t>
+        <v>50</v>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>4,7%</t>
+          <t>4,0%</t>
         </is>
       </c>
       <c r="L47" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>2,4%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
@@ -3917,12 +3917,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3947,33 +3947,33 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 135,00</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I48" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>16</v>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>▼ 27,3%</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>18,8%</t>
         </is>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>2,1%</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -3990,12 +3990,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4020,33 +4020,33 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>R$ 269,00</t>
+          <t>R$ 79,00</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>▲ 19,6%</t>
+          <t>▼ 36,3%</t>
         </is>
       </c>
       <c r="I49" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>▼ 30,9%</t>
+        <v>0</v>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>7,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L49" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>2,4%</t>
+          <t>1,2%</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
@@ -4063,12 +4063,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4093,33 +4093,33 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I50" s="2" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>▼ 38,1%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L50" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -4136,12 +4136,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4166,33 +4166,33 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>R$ 225,00</t>
+          <t>R$ 124,00</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>▲ 25,0%</t>
+          <t>▼ 44,9%</t>
         </is>
       </c>
       <c r="I51" s="2" t="n">
-        <v>123</v>
+        <v>61</v>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>▲ 23,0%</t>
+          <t>▼ 29,1%</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>4,1%</t>
+          <t>4,9%</t>
         </is>
       </c>
       <c r="L51" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>2,1%</t>
+          <t>1,3%</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
@@ -4209,12 +4209,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4244,20 +4244,20 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>▲ 61,5%</t>
+          <t>▼ 15,4%</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>9,1%</t>
         </is>
       </c>
       <c r="L52" s="2" t="n">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
@@ -4282,12 +4282,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4312,25 +4312,25 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>R$ 180,00</t>
+          <t>R$ 225,00</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>▲ 33,3%</t>
+          <t>▼ 16,4%</t>
         </is>
       </c>
       <c r="I53" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>▲ 25,0%</t>
+        <v>86</v>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>▲ 1,2%</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>4,0%</t>
+          <t>4,7%</t>
         </is>
       </c>
       <c r="L53" s="2" t="n">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>1,5%</t>
+          <t>2,4%</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
@@ -4355,12 +4355,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4385,33 +4385,33 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J54" s="4" t="inlineStr">
-        <is>
-          <t>▼ 48,0%</t>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L54" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
@@ -4428,12 +4428,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -4458,33 +4458,33 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>R$ 135,00</t>
+          <t>R$ 269,00</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>▼ 62,4%</t>
+          <t>▲ 19,6%</t>
         </is>
       </c>
       <c r="I55" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>▼ 23,1%</t>
+        <v>85</v>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>▼ 30,9%</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>3,8%</t>
+          <t>7,1%</t>
         </is>
       </c>
       <c r="L55" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>2,1%</t>
+          <t>2,4%</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
@@ -4501,12 +4501,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -4531,38 +4531,38 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>R$ 135,00</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>▲ 50,0%</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>▲ 19,0%</t>
+          <t>▼ 38,1%</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>12,0%</t>
+          <t>7,7%</t>
         </is>
       </c>
       <c r="L56" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>1,7%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O56" s="2" t="inlineStr">
@@ -4574,12 +4574,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -4604,33 +4604,33 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>R$ 359,00</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>▲ 697,8%</t>
+          <t>R$ 225,00</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>▲ 25,0%</t>
         </is>
       </c>
       <c r="I57" s="2" t="n">
-        <v>104</v>
-      </c>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t>▲ 42,5%</t>
+        <v>123</v>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>▲ 23,0%</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>4,1%</t>
         </is>
       </c>
       <c r="L57" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>2,1%</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr">
@@ -4647,12 +4647,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4677,33 +4677,33 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>▲ 50,0%</t>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>▲ 61,5%</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>9,5%</t>
+          <t>4,8%</t>
         </is>
       </c>
       <c r="L58" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -4720,12 +4720,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4750,33 +4750,33 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
+          <t>R$ 180,00</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>▼ 83,3%</t>
+          <t>▲ 33,3%</t>
         </is>
       </c>
       <c r="I59" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>▲ 43,1%</t>
+        <v>100</v>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>▲ 25,0%</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>1,4%</t>
+          <t>4,0%</t>
         </is>
       </c>
       <c r="L59" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>1,5%</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
@@ -4793,12 +4793,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4826,22 +4826,22 @@
           <t>R$ 45,00</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t>▼ 12,5%</t>
+        <v>13</v>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>▼ 48,0%</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>7,1%</t>
+          <t>7,7%</t>
         </is>
       </c>
       <c r="L60" s="2" t="n">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>0,6%</t>
+          <t>0,7%</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -4866,12 +4866,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -4896,33 +4896,33 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>R$ 269,00</t>
+          <t>R$ 135,00</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>▲ 198,9%</t>
+          <t>▼ 62,4%</t>
         </is>
       </c>
       <c r="I61" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>▼ 13,6%</t>
+        <v>80</v>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>▼ 23,1%</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>11,8%</t>
+          <t>3,8%</t>
         </is>
       </c>
       <c r="L61" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>3,6%</t>
+          <t>2,1%</t>
         </is>
       </c>
       <c r="N61" s="2" t="inlineStr">
@@ -4939,12 +4939,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4969,38 +4969,38 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 135,00</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>▲ 50,0%</t>
         </is>
       </c>
       <c r="I62" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="J62" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>25</v>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>▲ 19,0%</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>6,3%</t>
+          <t>12,0%</t>
         </is>
       </c>
       <c r="L62" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>1,7%</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
@@ -5012,12 +5012,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -5042,33 +5042,33 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 359,00</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>▲ 697,8%</t>
         </is>
       </c>
       <c r="I63" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>▲ 5,4%</t>
+        <v>104</v>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>▲ 42,5%</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>3,4%</t>
+          <t>7,7%</t>
         </is>
       </c>
       <c r="L63" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>0,9%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -5085,12 +5085,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -5115,38 +5115,38 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
+          <t>R$ 90,00</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="I64" s="2" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
-          <t>▼ 66,7%</t>
+          <t>▲ 50,0%</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>12,5%</t>
+          <t>9,5%</t>
         </is>
       </c>
       <c r="L64" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
@@ -5158,12 +5158,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -5188,33 +5188,33 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>▼ 83,3%</t>
         </is>
       </c>
       <c r="I65" s="2" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t>▼ 5,1%</t>
+          <t>▲ 43,1%</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>3,6%</t>
+          <t>1,4%</t>
         </is>
       </c>
       <c r="L65" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>0,9%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -5231,12 +5231,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -5261,38 +5261,38 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>▲ 300,0%</t>
+          <t>▼ 12,5%</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>8,3%</t>
+          <t>7,1%</t>
         </is>
       </c>
       <c r="L66" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr">
@@ -5304,12 +5304,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -5334,33 +5334,33 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>R$ 90,00</t>
+          <t>R$ 269,00</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▲ 198,9%</t>
         </is>
       </c>
       <c r="I67" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>▼ 3,3%</t>
+        <v>51</v>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>▼ 13,6%</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>3,4%</t>
+          <t>11,8%</t>
         </is>
       </c>
       <c r="L67" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>3,6%</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -5377,12 +5377,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5412,20 +5412,20 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="I68" s="2" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>▼ 40,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>16,7%</t>
+          <t>6,3%</t>
         </is>
       </c>
       <c r="L68" s="2" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
@@ -5450,12 +5450,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -5480,33 +5480,33 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>R$ 180,00</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+          <t>R$ 90,00</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I69" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="J69" s="3" t="inlineStr">
-        <is>
-          <t>▲ 56,4%</t>
+        <v>59</v>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>▲ 5,4%</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>6,6%</t>
+          <t>3,4%</t>
         </is>
       </c>
       <c r="L69" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>2,1%</t>
+          <t>0,9%</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr">
@@ -5523,12 +5523,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -5553,38 +5553,38 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="I70" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>▲ 42,9%</t>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>12,5%</t>
         </is>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr">
@@ -5596,12 +5596,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -5629,22 +5629,22 @@
           <t>R$ 90,00</t>
         </is>
       </c>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="I71" s="2" t="n">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>▲ 5,4%</t>
+          <t>▼ 5,1%</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>5,1%</t>
+          <t>3,6%</t>
         </is>
       </c>
       <c r="L71" s="2" t="n">
@@ -5669,12 +5669,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -5699,38 +5699,38 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 90,00</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>▼ 46,2%</t>
+          <t>▲ 300,0%</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>8,3%</t>
         </is>
       </c>
       <c r="L72" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
@@ -5742,12 +5742,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -5772,33 +5772,33 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>R$ 135,00</t>
+          <t>R$ 90,00</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>▲ 200,0%</t>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="J73" s="4" t="inlineStr">
-        <is>
-          <t>▼ 32,7%</t>
+        <v>59</v>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>▼ 3,3%</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>8,1%</t>
+          <t>3,4%</t>
         </is>
       </c>
       <c r="L73" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>1,8%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
@@ -5815,12 +5815,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -5850,20 +5850,20 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I74" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="J74" s="4" t="inlineStr">
-        <is>
-          <t>▼ 38,1%</t>
+        <v>6</v>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>▼ 40,0%</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>16,7%</t>
         </is>
       </c>
       <c r="L74" s="2" t="n">
@@ -5888,12 +5888,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -5918,33 +5918,33 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
+          <t>R$ 180,00</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>▼ 66,7%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="I75" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="J75" s="3" t="inlineStr">
-        <is>
-          <t>▲ 41,0%</t>
+        <v>61</v>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>▲ 56,4%</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>1,8%</t>
+          <t>6,6%</t>
         </is>
       </c>
       <c r="L75" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>2,1%</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
@@ -5961,12 +5961,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>R$ 45,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -6000,24 +6000,24 @@
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>10</v>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>▲ 42,9%</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L76" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
@@ -6034,12 +6034,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -6064,48 +6064,486 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>R$ 135,00</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 90,00</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="I77" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="J77" s="2" t="inlineStr">
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>▲ 5,4%</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>5,1%</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>0,9%</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-001</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Bingo 48 cartelas</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>1856971226</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>R$ 44,90</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>▼ 46,2%</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-001</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Bingo 48 cartelas</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>6167963928</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>R$ 44,90</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>R$ 135,00</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>▼ 32,7%</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>8,1%</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>1,8%</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-001</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Bingo 48 cartelas</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>1856971226</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>R$ 44,90</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>▼ 38,1%</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>7,7%</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>0,5%</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-001</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Bingo 48 cartelas</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>6167963928</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>R$ 44,90</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>▲ 41,0%</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>1,8%</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>0,5%</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-001</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Bingo 48 cartelas</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>1856971226</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>R$ 44,90</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>R$ 45,00</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K77" s="2" t="inlineStr">
+      <c r="I82" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>4,8%</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>0,5%</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-001</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Bingo 48 cartelas</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>6167963928</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>R$ 44,90</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>R$ 135,00</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
         <is>
           <t>7,7%</t>
         </is>
       </c>
-      <c r="L77" s="2" t="n">
+      <c r="L83" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M77" s="2" t="inlineStr">
+      <c r="M83" s="2" t="inlineStr">
         <is>
           <t>1,5%</t>
         </is>
       </c>
-      <c r="N77" s="2" t="inlineStr">
+      <c r="N83" s="2" t="inlineStr">
         <is>
           <t>Sem calcular</t>
         </is>
       </c>
-      <c r="O77" s="2" t="inlineStr">
+      <c r="O83" s="2" t="inlineStr">
         <is>
           <t>Boa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O77"/>
+  <autoFilter ref="A1:O83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>